<commit_message>
Aggregate statistics to the state level
</commit_message>
<xml_diff>
--- a/a_in/us_travels.xlsx
+++ b/a_in/us_travels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/s9/Code/us_travels_v4/a_in/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90A4B47A-63CC-5F42-9A01-335BECC967F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DBFB445-6AD9-4E4C-9F65-A17DACA157E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38840" yWindow="800" windowWidth="34120" windowHeight="20100" activeTab="3" xr2:uid="{895BEAD3-490B-3645-811C-E95312094DBD}"/>
+    <workbookView xWindow="9800" yWindow="660" windowWidth="23040" windowHeight="21680" activeTab="1" xr2:uid="{895BEAD3-490B-3645-811C-E95312094DBD}"/>
   </bookViews>
   <sheets>
     <sheet name="area_region" sheetId="4" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3511" uniqueCount="1199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3512" uniqueCount="1200">
   <si>
     <t>New York–Newark–Jersey City, NY-NJ MSA</t>
   </si>
@@ -3642,6 +3642,9 @@
   </si>
   <si>
     <t>Augusta, ME µsa</t>
+  </si>
+  <si>
+    <t>metro_population</t>
   </si>
 </sst>
 </file>
@@ -3742,7 +3745,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="15" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -3775,6 +3778,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -5696,7 +5700,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A7F6F74-518A-5046-A708-32A1E165FF17}">
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
@@ -5705,9 +5709,10 @@
     <col min="4" max="4" width="8.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>587</v>
       </c>
@@ -5726,8 +5731,11 @@
       <c r="F1" s="1" t="s">
         <v>1127</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G1" s="1" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>701</v>
       </c>
@@ -5747,8 +5755,11 @@
       <c r="F2" s="1" t="s">
         <v>737</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G2" s="22">
+        <v>534419</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>628</v>
       </c>
@@ -5768,8 +5779,11 @@
       <c r="F3" s="1" t="s">
         <v>708</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G3" s="22">
+        <v>3975019</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>667</v>
       </c>
@@ -5789,8 +5803,11 @@
       <c r="F4" s="1" t="s">
         <v>847</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4" s="22">
+        <v>1845775</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>605</v>
       </c>
@@ -5810,8 +5827,11 @@
       <c r="F5" s="1" t="s">
         <v>559</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G5" s="22">
+        <v>7236843</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>589</v>
       </c>
@@ -5831,8 +5851,11 @@
       <c r="F6" s="1" t="s">
         <v>576</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G6" s="22">
+        <v>38588946</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>613</v>
       </c>
@@ -5852,8 +5875,11 @@
       <c r="F7" s="1" t="s">
         <v>568</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G7" s="22">
+        <v>5235839</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>632</v>
       </c>
@@ -5873,8 +5899,11 @@
       <c r="F8" s="1" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G8" s="22">
+        <v>3463267</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>609</v>
       </c>
@@ -5894,8 +5923,11 @@
       <c r="F9" s="1" t="s">
         <v>556</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G9" s="22">
+        <v>6436489</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>722</v>
       </c>
@@ -5915,8 +5947,11 @@
       <c r="F10" s="1" t="s">
         <v>723</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G10" s="22">
+        <v>192690</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>608</v>
       </c>
@@ -5936,8 +5971,11 @@
       <c r="F11" s="1" t="s">
         <v>709</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G11" s="22">
+        <v>22683498</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>603</v>
       </c>
@@ -5957,8 +5995,11 @@
       <c r="F12" s="1" t="s">
         <v>557</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G12" s="22">
+        <v>9442998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>640</v>
       </c>
@@ -5978,8 +6019,11 @@
       <c r="F13" s="1" t="s">
         <v>639</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G13" s="22">
+        <v>1162516</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>670</v>
       </c>
@@ -5999,8 +6043,11 @@
       <c r="F14" s="1" t="s">
         <v>669</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G14" s="22">
+        <v>2141646</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>662</v>
       </c>
@@ -6020,8 +6067,11 @@
       <c r="F15" s="1" t="s">
         <v>661</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G15" s="22">
+        <v>1484378</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>590</v>
       </c>
@@ -6041,8 +6091,11 @@
       <c r="F16" s="1" t="s">
         <v>720</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G16" s="22">
+        <v>10938221</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>620</v>
       </c>
@@ -6062,8 +6115,11 @@
       <c r="F17" s="1" t="s">
         <v>582</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G17" s="22">
+        <v>4396584</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>677</v>
       </c>
@@ -6083,8 +6139,11 @@
       <c r="F18" s="1" t="s">
         <v>717</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G18" s="22">
+        <v>1150746</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>626</v>
       </c>
@@ -6104,8 +6163,11 @@
       <c r="F19" s="1" t="s">
         <v>738</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G19" s="22">
+        <v>2495293</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>645</v>
       </c>
@@ -6125,8 +6187,11 @@
       <c r="F20" s="1" t="s">
         <v>654</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G20" s="22">
+        <v>3881403</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>606</v>
       </c>
@@ -6146,8 +6211,11 @@
       <c r="F21" s="1" t="s">
         <v>560</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G21" s="22">
+        <v>6897611</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>615</v>
       </c>
@@ -6167,8 +6235,11 @@
       <c r="F22" s="1" t="s">
         <v>740</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G22" s="22">
+        <v>3554083</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>693</v>
       </c>
@@ -6188,8 +6259,11 @@
       <c r="F23" s="1" t="s">
         <v>739</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G23" s="22">
+        <v>862535</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>610</v>
       </c>
@@ -6209,8 +6283,11 @@
       <c r="F24" s="1" t="s">
         <v>741</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G24" s="22">
+        <v>8411524</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>612</v>
       </c>
@@ -6230,8 +6307,11 @@
       <c r="F25" s="1" t="s">
         <v>565</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G25" s="22">
+        <v>4581580</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>616</v>
       </c>
@@ -6251,8 +6331,11 @@
       <c r="F26" s="1" t="s">
         <v>727</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G26" s="22">
+        <v>6358547</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>684</v>
       </c>
@@ -6272,8 +6355,11 @@
       <c r="F27" s="1" t="s">
         <v>683</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G27" s="22">
+        <v>1189546</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>724</v>
       </c>
@@ -6293,8 +6379,11 @@
       <c r="F28" s="1" t="s">
         <v>730</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G28" s="22">
+        <v>628514</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>614</v>
       </c>
@@ -6314,8 +6403,11 @@
       <c r="F29" s="1" t="s">
         <v>596</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G29" s="22">
+        <v>9194154</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>715</v>
       </c>
@@ -6335,8 +6427,11 @@
       <c r="F30" s="1" t="s">
         <v>728</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G30" s="22">
+        <v>587098</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>638</v>
       </c>
@@ -6356,8 +6451,11 @@
       <c r="F31" s="1" t="s">
         <v>707</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G31" s="22">
+        <v>1428914</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>699</v>
       </c>
@@ -6377,8 +6475,11 @@
       <c r="F32" s="1" t="s">
         <v>742</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G32" s="22">
+        <v>474438</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>703</v>
       </c>
@@ -6398,8 +6499,11 @@
       <c r="F33" s="1" t="s">
         <v>704</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G33" s="22">
+        <v>1014680</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>649</v>
       </c>
@@ -6419,8 +6523,11 @@
       <c r="F34" s="1" t="s">
         <v>726</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G34" s="22">
+        <v>1434251</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>618</v>
       </c>
@@ -6440,8 +6547,11 @@
       <c r="F35" s="1" t="s">
         <v>729</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G35" s="22">
+        <v>3032129</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>588</v>
       </c>
@@ -6461,8 +6571,11 @@
       <c r="F36" s="1" t="s">
         <v>652</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G36" s="22">
+        <v>25577932</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>619</v>
       </c>
@@ -6482,8 +6595,11 @@
       <c r="F37" s="1" t="s">
         <v>581</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G37" s="22">
+        <v>10126288</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>625</v>
       </c>
@@ -6503,8 +6619,11 @@
       <c r="F38" s="1" t="s">
         <v>597</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G38" s="22">
+        <v>2746530</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>617</v>
       </c>
@@ -6524,8 +6643,11 @@
       <c r="F39" s="1" t="s">
         <v>710</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G39" s="22">
+        <v>4169103</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>604</v>
       </c>
@@ -6545,8 +6667,11 @@
       <c r="F40" s="1" t="s">
         <v>682</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G40" s="22">
+        <v>13513463</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>734</v>
       </c>
@@ -6566,8 +6691,11 @@
       <c r="F41" s="1" t="s">
         <v>733</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G41" s="22">
+        <v>2035484</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>623</v>
       </c>
@@ -6587,8 +6715,11 @@
       <c r="F42" s="1" t="s">
         <v>594</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G42" s="22">
+        <v>1700901</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>642</v>
       </c>
@@ -6608,8 +6739,11 @@
       <c r="F43" s="1" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G43" s="22">
+        <v>4088781</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>712</v>
       </c>
@@ -6629,8 +6763,11 @@
       <c r="F44" s="1" t="s">
         <v>743</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G44" s="22">
+        <v>478584</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>621</v>
       </c>
@@ -6650,8 +6787,11 @@
       <c r="F45" s="1" t="s">
         <v>584</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G45" s="22">
+        <v>6353067</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>607</v>
       </c>
@@ -6671,8 +6811,11 @@
       <c r="F46" s="1" t="s">
         <v>574</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G46" s="22">
+        <v>28360769</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>627</v>
       </c>
@@ -6692,8 +6835,11 @@
       <c r="F47" s="1" t="s">
         <v>601</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G47" s="22">
+        <v>3098042</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>622</v>
       </c>
@@ -6713,8 +6859,11 @@
       <c r="F48" s="1" t="s">
         <v>599</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G48" s="22">
+        <v>4573022</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>718</v>
       </c>
@@ -6734,8 +6883,11 @@
       <c r="F49" s="1" t="s">
         <v>744</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G49" s="22">
+        <v>237519</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>611</v>
       </c>
@@ -6755,8 +6907,11 @@
       <c r="F50" s="1" t="s">
         <v>714</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G50" s="22">
+        <v>6583502</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>624</v>
       </c>
@@ -6776,8 +6931,11 @@
       <c r="F51" s="1" t="s">
         <v>673</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G51" s="22">
+        <v>4280527</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>705</v>
       </c>
@@ -6797,8 +6955,11 @@
       <c r="F52" s="1" t="s">
         <v>721</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G52" s="22">
+        <v>1158798</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>731</v>
       </c>
@@ -6817,6 +6978,9 @@
       </c>
       <c r="F53" s="1" t="s">
         <v>732</v>
+      </c>
+      <c r="G53" s="22">
+        <v>182193</v>
       </c>
     </row>
   </sheetData>
@@ -16620,7 +16784,7 @@
         <v>624</v>
       </c>
       <c r="C386" s="19">
-        <f t="shared" ref="C386:C449" si="6">INT(NOT(AND(ISBLANK(D386),ISBLANK(E386),ISBLANK(F386),ISBLANK(G386))))</f>
+        <f t="shared" ref="C386:C397" si="6">INT(NOT(AND(ISBLANK(D386),ISBLANK(E386),ISBLANK(F386),ISBLANK(G386))))</f>
         <v>0</v>
       </c>
       <c r="D386" s="5"/>

</xml_diff>